<commit_message>
dgft and customs excel and pdf dgft
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CUSTOMS_EXCEL/Acts/Customs Act, 1962.xlsx
+++ b/backend/PDF_DOC/CUSTOMS_EXCEL/Acts/Customs Act, 1962.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4961E5-B68E-48F1-B8F9-EE4C744F2136}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4961E5-B68E-48F1-B8F9-EE4C744F2136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="18" activeTab="27" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="18" activeTab="27" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CHAPTER 1" sheetId="1" r:id="rId1"/>
@@ -8928,14 +8928,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -9389,12 +9387,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>17</v>
       </c>
@@ -9925,7 +9923,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>790</v>
       </c>
     </row>
@@ -13453,7 +13451,7 @@
       <c r="A122" t="s">
         <v>1259</v>
       </c>
-      <c r="B122" s="4" t="s">
+      <c r="B122" t="s">
         <v>1260</v>
       </c>
     </row>
@@ -15011,7 +15009,7 @@
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>1501</v>
       </c>
@@ -15127,7 +15125,7 @@
       <c r="A4" s="1" t="s">
         <v>1514</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>1515</v>
       </c>
     </row>
@@ -15520,7 +15518,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>120</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -16053,10 +16051,10 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>1620</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>1621</v>
       </c>
     </row>
@@ -26385,12 +26383,12 @@
   <dimension ref="A1:B59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>198</v>
       </c>
     </row>
@@ -26549,12 +26547,12 @@
   <dimension ref="A1:B81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="128" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>263</v>
       </c>
     </row>
@@ -26706,7 +26704,7 @@
       </c>
     </row>
     <row r="47" spans="1:2" ht="90" x14ac:dyDescent="0.25">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="3" t="s">
         <v>252</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -26727,7 +26725,7 @@
       </c>
     </row>
     <row r="54" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="3" t="s">
         <v>256</v>
       </c>
       <c r="B54" s="1" t="s">
@@ -26818,7 +26816,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>298</v>
       </c>
     </row>
@@ -27005,7 +27003,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>299</v>
       </c>
     </row>
@@ -27040,12 +27038,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>305</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -27054,103 +27052,87 @@
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
       <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
       <c r="B6" s="1" t="s">
         <v>307</v>
       </c>
       <c r="C6" s="1"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
       <c r="C7" s="1"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
       <c r="B8" s="1" t="s">
         <v>308</v>
       </c>
       <c r="C8" s="1"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
       <c r="B10" s="1" t="s">
         <v>309</v>
       </c>
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-    </row>
     <row r="13" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" t="s">
         <v>310</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-    </row>
     <row r="16" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" t="s">
         <v>312</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
-    </row>
-    <row r="18" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" ht="60" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:2" ht="45" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:2" ht="45" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>317</v>
       </c>
@@ -27198,9 +27180,6 @@
         <v>330</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="4"/>
-    </row>
     <row r="51" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B51" s="1" t="s">
         <v>331</v>
@@ -27269,9 +27248,6 @@
         <v>344</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="4"/>
-    </row>
     <row r="80" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B80" s="1" t="s">
         <v>345</v>
@@ -27293,7 +27269,7 @@
       </c>
     </row>
     <row r="90" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A90" s="4" t="s">
+      <c r="A90" t="s">
         <v>364</v>
       </c>
       <c r="B90" s="1" t="s">
@@ -27412,9 +27388,6 @@
       <c r="B135" s="1" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" s="4"/>
     </row>
     <row r="137" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B137" s="1" t="s">
@@ -29496,7 +29469,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>783</v>
       </c>
     </row>
@@ -29504,7 +29477,7 @@
       <c r="A4" s="1" t="s">
         <v>784</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>785</v>
       </c>
     </row>

</xml_diff>